<commit_message>
gestion de la colonne province dans IREP
</commit_message>
<xml_diff>
--- a/data/RDC_Zone_de_sante_OCHA.xlsx
+++ b/data/RDC_Zone_de_sante_OCHA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Benjamin MUPANZI\Documents\incident_dashboard\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{255B0FA6-6732-4CDB-9022-C594E452F129}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DBAE1F0-126D-43E2-AA13-ED701468B4D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6709,12 +6709,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I520"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1024" width="15"/>
+    <col min="1" max="1" width="15"/>
+    <col min="2" max="2" width="32.7109375" customWidth="1"/>
+    <col min="3" max="1024" width="15"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -6743,7 +6745,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -6772,7 +6774,7 @@
         <v>24.67352606</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -6801,7 +6803,7 @@
         <v>22.263098079999999</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -6830,7 +6832,7 @@
         <v>23.836046110000002</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -6859,7 +6861,7 @@
         <v>24.12357166</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -6888,7 +6890,7 @@
         <v>23.322223999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -6917,7 +6919,7 @@
         <v>24.238741300000001</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -6946,7 +6948,7 @@
         <v>23.453407439999999</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -6975,7 +6977,7 @@
         <v>23.51581771</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -7004,7 +7006,7 @@
         <v>23.38849063</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -7033,7 +7035,7 @@
         <v>24.119463020000001</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -7062,7 +7064,7 @@
         <v>24.73568684</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -7091,7 +7093,7 @@
         <v>22.74943094</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>9</v>
       </c>
@@ -7120,7 +7122,7 @@
         <v>23.223269729999998</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>9</v>
       </c>
@@ -7149,7 +7151,7 @@
         <v>23.738399399999999</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>9</v>
       </c>
@@ -7178,7 +7180,7 @@
         <v>23.337240640000001</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>9</v>
       </c>
@@ -7207,7 +7209,7 @@
         <v>24.047591449999999</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>9</v>
       </c>
@@ -7236,7 +7238,7 @@
         <v>23.86608888</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>9</v>
       </c>
@@ -7265,7 +7267,7 @@
         <v>23.706285730000001</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>9</v>
       </c>
@@ -7294,7 +7296,7 @@
         <v>23.293699199999999</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>9</v>
       </c>
@@ -7323,7 +7325,7 @@
         <v>25.878419099999999</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>9</v>
       </c>
@@ -7352,7 +7354,7 @@
         <v>25.096385430000002</v>
       </c>
     </row>
-    <row r="23" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>9</v>
       </c>
@@ -7381,7 +7383,7 @@
         <v>24.440722180000002</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>9</v>
       </c>
@@ -7410,7 +7412,7 @@
         <v>24.49348213</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>9</v>
       </c>
@@ -7439,7 +7441,7 @@
         <v>24.409599069999999</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>9</v>
       </c>
@@ -7468,7 +7470,7 @@
         <v>23.41709419</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>9</v>
       </c>
@@ -7497,7 +7499,7 @@
         <v>23.413497620000001</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>9</v>
       </c>
@@ -7526,7 +7528,7 @@
         <v>23.313230319999999</v>
       </c>
     </row>
-    <row r="29" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>9</v>
       </c>
@@ -7555,7 +7557,7 @@
         <v>23.784982540000001</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>9</v>
       </c>
@@ -7584,7 +7586,7 @@
         <v>23.751760239999999</v>
       </c>
     </row>
-    <row r="31" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>9</v>
       </c>
@@ -7613,7 +7615,7 @@
         <v>23.612171660000001</v>
       </c>
     </row>
-    <row r="32" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>9</v>
       </c>
@@ -7642,7 +7644,7 @@
         <v>23.619222350000001</v>
       </c>
     </row>
-    <row r="33" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>9</v>
       </c>
@@ -7671,7 +7673,7 @@
         <v>23.609278079999999</v>
       </c>
     </row>
-    <row r="34" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>9</v>
       </c>
@@ -7700,7 +7702,7 @@
         <v>23.633013800000001</v>
       </c>
     </row>
-    <row r="35" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>9</v>
       </c>
@@ -7729,7 +7731,7 @@
         <v>23.598031639999999</v>
       </c>
     </row>
-    <row r="36" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>9</v>
       </c>
@@ -7758,7 +7760,7 @@
         <v>23.573470499999999</v>
       </c>
     </row>
-    <row r="37" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>9</v>
       </c>
@@ -7787,7 +7789,7 @@
         <v>23.543476429999998</v>
       </c>
     </row>
-    <row r="38" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>9</v>
       </c>
@@ -7816,7 +7818,7 @@
         <v>23.550350359999999</v>
       </c>
     </row>
-    <row r="39" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>9</v>
       </c>
@@ -7845,7 +7847,7 @@
         <v>23.16772319</v>
       </c>
     </row>
-    <row r="40" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>9</v>
       </c>
@@ -7874,7 +7876,7 @@
         <v>23.58956147</v>
       </c>
     </row>
-    <row r="41" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>9</v>
       </c>
@@ -7903,7 +7905,7 @@
         <v>23.651351259999998</v>
       </c>
     </row>
-    <row r="42" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>9</v>
       </c>
@@ -7932,7 +7934,7 @@
         <v>23.485315809999999</v>
       </c>
     </row>
-    <row r="43" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>9</v>
       </c>
@@ -7961,7 +7963,7 @@
         <v>23.610476640000002</v>
       </c>
     </row>
-    <row r="44" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>9</v>
       </c>
@@ -7990,7 +7992,7 @@
         <v>25.397675320000001</v>
       </c>
     </row>
-    <row r="45" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>9</v>
       </c>
@@ -8019,7 +8021,7 @@
         <v>23.615871739999999</v>
       </c>
     </row>
-    <row r="46" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>9</v>
       </c>
@@ -8048,7 +8050,7 @@
         <v>23.910934520000001</v>
       </c>
     </row>
-    <row r="47" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>9</v>
       </c>
@@ -8077,7 +8079,7 @@
         <v>23.447657790000001</v>
       </c>
     </row>
-    <row r="48" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>9</v>
       </c>
@@ -8106,7 +8108,7 @@
         <v>24.993487179999999</v>
       </c>
     </row>
-    <row r="49" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>9</v>
       </c>
@@ -8135,7 +8137,7 @@
         <v>21.1391907</v>
       </c>
     </row>
-    <row r="50" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>9</v>
       </c>
@@ -8164,7 +8166,7 @@
         <v>20.382563449999999</v>
       </c>
     </row>
-    <row r="51" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>9</v>
       </c>
@@ -8193,7 +8195,7 @@
         <v>20.844926539999999</v>
       </c>
     </row>
-    <row r="52" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>9</v>
       </c>
@@ -8222,7 +8224,7 @@
         <v>20.899172709999998</v>
       </c>
     </row>
-    <row r="53" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>9</v>
       </c>
@@ -8251,7 +8253,7 @@
         <v>21.384131010000001</v>
       </c>
     </row>
-    <row r="54" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>9</v>
       </c>
@@ -8280,7 +8282,7 @@
         <v>20.528917790000001</v>
       </c>
     </row>
-    <row r="55" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>9</v>
       </c>
@@ -8309,7 +8311,7 @@
         <v>21.317013209999999</v>
       </c>
     </row>
-    <row r="56" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>9</v>
       </c>
@@ -8338,7 +8340,7 @@
         <v>21.605729409999999</v>
       </c>
     </row>
-    <row r="57" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>9</v>
       </c>
@@ -8367,7 +8369,7 @@
         <v>29.988244099999999</v>
       </c>
     </row>
-    <row r="58" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>9</v>
       </c>
@@ -8396,7 +8398,7 @@
         <v>19.727392890000001</v>
       </c>
     </row>
-    <row r="59" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>9</v>
       </c>
@@ -8425,7 +8427,7 @@
         <v>12.497372800000001</v>
       </c>
     </row>
-    <row r="60" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>9</v>
       </c>
@@ -8454,7 +8456,7 @@
         <v>12.442850679999999</v>
       </c>
     </row>
-    <row r="61" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>9</v>
       </c>
@@ -8483,7 +8485,7 @@
         <v>13.0534888</v>
       </c>
     </row>
-    <row r="62" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>9</v>
       </c>
@@ -8512,7 +8514,7 @@
         <v>12.974744749999999</v>
       </c>
     </row>
-    <row r="63" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>9</v>
       </c>
@@ -8541,7 +8543,7 @@
         <v>13.28573445</v>
       </c>
     </row>
-    <row r="64" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>9</v>
       </c>
@@ -8570,7 +8572,7 @@
         <v>13.47696421</v>
       </c>
     </row>
-    <row r="65" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>9</v>
       </c>
@@ -8599,7 +8601,7 @@
         <v>12.82912917</v>
       </c>
     </row>
-    <row r="66" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>9</v>
       </c>
@@ -8628,7 +8630,7 @@
         <v>12.89115002</v>
       </c>
     </row>
-    <row r="67" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>9</v>
       </c>
@@ -8657,7 +8659,7 @@
         <v>13.01121215</v>
       </c>
     </row>
-    <row r="68" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>9</v>
       </c>
@@ -8686,7 +8688,7 @@
         <v>12.960746820000001</v>
       </c>
     </row>
-    <row r="69" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>9</v>
       </c>
@@ -8715,7 +8717,7 @@
         <v>13.67157282</v>
       </c>
     </row>
-    <row r="70" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>9</v>
       </c>
@@ -8744,7 +8746,7 @@
         <v>13.93446136</v>
       </c>
     </row>
-    <row r="71" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>9</v>
       </c>
@@ -8773,7 +8775,7 @@
         <v>14.92004712</v>
       </c>
     </row>
-    <row r="72" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>9</v>
       </c>
@@ -8802,7 +8804,7 @@
         <v>15.50528506</v>
       </c>
     </row>
-    <row r="73" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>9</v>
       </c>
@@ -8831,7 +8833,7 @@
         <v>15.016526430000001</v>
       </c>
     </row>
-    <row r="74" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>9</v>
       </c>
@@ -8860,7 +8862,7 @@
         <v>14.80878581</v>
       </c>
     </row>
-    <row r="75" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>9</v>
       </c>
@@ -8889,7 +8891,7 @@
         <v>14.64259283</v>
       </c>
     </row>
-    <row r="76" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>9</v>
       </c>
@@ -8918,7 +8920,7 @@
         <v>15.282318549999999</v>
       </c>
     </row>
-    <row r="77" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>9</v>
       </c>
@@ -8947,7 +8949,7 @@
         <v>20.548836390000002</v>
       </c>
     </row>
-    <row r="78" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>9</v>
       </c>
@@ -8976,7 +8978,7 @@
         <v>20.044599059999999</v>
       </c>
     </row>
-    <row r="79" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>9</v>
       </c>
@@ -9005,7 +9007,7 @@
         <v>19.192332889999999</v>
       </c>
     </row>
-    <row r="80" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>9</v>
       </c>
@@ -9034,7 +9036,7 @@
         <v>18.621061040000001</v>
       </c>
     </row>
-    <row r="81" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>9</v>
       </c>
@@ -9063,7 +9065,7 @@
         <v>17.821123979999999</v>
       </c>
     </row>
-    <row r="82" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>9</v>
       </c>
@@ -9092,7 +9094,7 @@
         <v>17.909069379999998</v>
       </c>
     </row>
-    <row r="83" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>9</v>
       </c>
@@ -9121,7 +9123,7 @@
         <v>19.454103780000001</v>
       </c>
     </row>
-    <row r="84" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>9</v>
       </c>
@@ -9150,7 +9152,7 @@
         <v>19.709546929999998</v>
       </c>
     </row>
-    <row r="85" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>9</v>
       </c>
@@ -9179,7 +9181,7 @@
         <v>19.89091561</v>
       </c>
     </row>
-    <row r="86" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>9</v>
       </c>
@@ -9208,7 +9210,7 @@
         <v>18.633765289999999</v>
       </c>
     </row>
-    <row r="87" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>9</v>
       </c>
@@ -9237,7 +9239,7 @@
         <v>18.85961438</v>
       </c>
     </row>
-    <row r="88" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>9</v>
       </c>
@@ -9266,7 +9268,7 @@
         <v>17.848019270000002</v>
       </c>
     </row>
-    <row r="89" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>9</v>
       </c>
@@ -9295,7 +9297,7 @@
         <v>17.445192160000001</v>
       </c>
     </row>
-    <row r="90" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>9</v>
       </c>
@@ -9324,7 +9326,7 @@
         <v>18.509952689999999</v>
       </c>
     </row>
-    <row r="91" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
         <v>9</v>
       </c>
@@ -9353,7 +9355,7 @@
         <v>18.824129490000001</v>
       </c>
     </row>
-    <row r="92" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
         <v>9</v>
       </c>
@@ -9382,7 +9384,7 @@
         <v>18.91037983</v>
       </c>
     </row>
-    <row r="93" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
         <v>9</v>
       </c>
@@ -9411,7 +9413,7 @@
         <v>18.38306554</v>
       </c>
     </row>
-    <row r="94" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
         <v>9</v>
       </c>
@@ -9440,7 +9442,7 @@
         <v>17.324294680000001</v>
       </c>
     </row>
-    <row r="95" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
         <v>9</v>
       </c>
@@ -9469,7 +9471,7 @@
         <v>18.064585810000001</v>
       </c>
     </row>
-    <row r="96" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
         <v>9</v>
       </c>
@@ -9498,7 +9500,7 @@
         <v>17.693119849999999</v>
       </c>
     </row>
-    <row r="97" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>9</v>
       </c>
@@ -9527,7 +9529,7 @@
         <v>18.036671720000001</v>
       </c>
     </row>
-    <row r="98" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
         <v>9</v>
       </c>
@@ -9556,7 +9558,7 @@
         <v>17.252226719999999</v>
       </c>
     </row>
-    <row r="99" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
         <v>9</v>
       </c>
@@ -9585,7 +9587,7 @@
         <v>17.358020799999998</v>
       </c>
     </row>
-    <row r="100" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
         <v>9</v>
       </c>
@@ -9614,7 +9616,7 @@
         <v>16.734431010000002</v>
       </c>
     </row>
-    <row r="101" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
         <v>9</v>
       </c>
@@ -9643,7 +9645,7 @@
         <v>27.34589652</v>
       </c>
     </row>
-    <row r="102" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
         <v>9</v>
       </c>
@@ -9672,7 +9674,7 @@
         <v>26.700383720000001</v>
       </c>
     </row>
-    <row r="103" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
         <v>9</v>
       </c>
@@ -9701,7 +9703,7 @@
         <v>24.40886223</v>
       </c>
     </row>
-    <row r="104" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
         <v>9</v>
       </c>
@@ -9730,7 +9732,7 @@
         <v>23.747219959999999</v>
       </c>
     </row>
-    <row r="105" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
         <v>9</v>
       </c>
@@ -9759,7 +9761,7 @@
         <v>25.040651579999999</v>
       </c>
     </row>
-    <row r="106" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
         <v>9</v>
       </c>
@@ -9788,7 +9790,7 @@
         <v>24.63989273</v>
       </c>
     </row>
-    <row r="107" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
         <v>9</v>
       </c>
@@ -9817,7 +9819,7 @@
         <v>23.925672689999999</v>
       </c>
     </row>
-    <row r="108" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
         <v>9</v>
       </c>
@@ -9846,7 +9848,7 @@
         <v>23.975615940000001</v>
       </c>
     </row>
-    <row r="109" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
         <v>9</v>
       </c>
@@ -9875,7 +9877,7 @@
         <v>24.399625270000001</v>
       </c>
     </row>
-    <row r="110" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
         <v>9</v>
       </c>
@@ -9904,7 +9906,7 @@
         <v>24.635368849999999</v>
       </c>
     </row>
-    <row r="111" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
         <v>9</v>
       </c>
@@ -9933,7 +9935,7 @@
         <v>25.615560429999999</v>
       </c>
     </row>
-    <row r="112" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
         <v>9</v>
       </c>
@@ -9962,7 +9964,7 @@
         <v>26.690724970000002</v>
       </c>
     </row>
-    <row r="113" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
         <v>9</v>
       </c>
@@ -9991,7 +9993,7 @@
         <v>26.731261549999999</v>
       </c>
     </row>
-    <row r="114" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
         <v>9</v>
       </c>
@@ -10020,7 +10022,7 @@
         <v>24.979732930000001</v>
       </c>
     </row>
-    <row r="115" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
         <v>9</v>
       </c>
@@ -10049,7 +10051,7 @@
         <v>25.484702349999999</v>
       </c>
     </row>
-    <row r="116" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
         <v>9</v>
       </c>
@@ -10078,7 +10080,7 @@
         <v>25.972853990000001</v>
       </c>
     </row>
-    <row r="117" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
         <v>9</v>
       </c>
@@ -10107,7 +10109,7 @@
         <v>18.318667940000001</v>
       </c>
     </row>
-    <row r="118" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
         <v>9</v>
       </c>
@@ -10136,7 +10138,7 @@
         <v>18.615981600000001</v>
       </c>
     </row>
-    <row r="119" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
         <v>9</v>
       </c>
@@ -10165,7 +10167,7 @@
         <v>18.542584179999999</v>
       </c>
     </row>
-    <row r="120" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
         <v>9</v>
       </c>
@@ -10194,7 +10196,7 @@
         <v>19.074680669999999</v>
       </c>
     </row>
-    <row r="121" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
         <v>9</v>
       </c>
@@ -10223,7 +10225,7 @@
         <v>19.341847999999999</v>
       </c>
     </row>
-    <row r="122" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
         <v>9</v>
       </c>
@@ -10252,7 +10254,7 @@
         <v>18.191483160000001</v>
       </c>
     </row>
-    <row r="123" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
         <v>9</v>
       </c>
@@ -10281,7 +10283,7 @@
         <v>18.499046669999998</v>
       </c>
     </row>
-    <row r="124" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
         <v>9</v>
       </c>
@@ -10310,7 +10312,7 @@
         <v>13.469136499999999</v>
       </c>
     </row>
-    <row r="125" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
         <v>9</v>
       </c>
@@ -10339,7 +10341,7 @@
         <v>13.4087713</v>
       </c>
     </row>
-    <row r="126" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
         <v>9</v>
       </c>
@@ -10368,7 +10370,7 @@
         <v>15.37358699</v>
       </c>
     </row>
-    <row r="127" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A127" t="s">
         <v>9</v>
       </c>
@@ -10397,7 +10399,7 @@
         <v>15.298458009999999</v>
       </c>
     </row>
-    <row r="128" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
         <v>9</v>
       </c>
@@ -10426,7 +10428,7 @@
         <v>15.40239341</v>
       </c>
     </row>
-    <row r="129" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A129" t="s">
         <v>9</v>
       </c>
@@ -10455,7 +10457,7 @@
         <v>15.47441905</v>
       </c>
     </row>
-    <row r="130" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A130" t="s">
         <v>9</v>
       </c>
@@ -10484,7 +10486,7 @@
         <v>15.320750370000001</v>
       </c>
     </row>
-    <row r="131" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A131" t="s">
         <v>9</v>
       </c>
@@ -10513,7 +10515,7 @@
         <v>15.35044207</v>
       </c>
     </row>
-    <row r="132" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A132" t="s">
         <v>9</v>
       </c>
@@ -10542,7 +10544,7 @@
         <v>15.344765410000001</v>
       </c>
     </row>
-    <row r="133" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A133" t="s">
         <v>9</v>
       </c>
@@ -10571,7 +10573,7 @@
         <v>15.30079299</v>
       </c>
     </row>
-    <row r="134" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A134" t="s">
         <v>9</v>
       </c>
@@ -10600,7 +10602,7 @@
         <v>15.32536101</v>
       </c>
     </row>
-    <row r="135" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A135" t="s">
         <v>9</v>
       </c>
@@ -10629,7 +10631,7 @@
         <v>15.31190473</v>
       </c>
     </row>
-    <row r="136" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A136" t="s">
         <v>9</v>
       </c>
@@ -10658,7 +10660,7 @@
         <v>15.336309869999999</v>
       </c>
     </row>
-    <row r="137" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A137" t="s">
         <v>9</v>
       </c>
@@ -10687,7 +10689,7 @@
         <v>15.319805179999999</v>
       </c>
     </row>
-    <row r="138" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A138" t="s">
         <v>9</v>
       </c>
@@ -10716,7 +10718,7 @@
         <v>15.315630499999999</v>
       </c>
     </row>
-    <row r="139" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A139" t="s">
         <v>9</v>
       </c>
@@ -10745,7 +10747,7 @@
         <v>15.29394469</v>
       </c>
     </row>
-    <row r="140" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A140" t="s">
         <v>9</v>
       </c>
@@ -10774,7 +10776,7 @@
         <v>15.308048899999999</v>
       </c>
     </row>
-    <row r="141" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A141" t="s">
         <v>9</v>
       </c>
@@ -10803,7 +10805,7 @@
         <v>15.322621440000001</v>
       </c>
     </row>
-    <row r="142" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A142" t="s">
         <v>9</v>
       </c>
@@ -10832,7 +10834,7 @@
         <v>15.28391165</v>
       </c>
     </row>
-    <row r="143" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A143" t="s">
         <v>9</v>
       </c>
@@ -10861,7 +10863,7 @@
         <v>15.277608470000001</v>
       </c>
     </row>
-    <row r="144" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A144" t="s">
         <v>9</v>
       </c>
@@ -10890,7 +10892,7 @@
         <v>15.41615008</v>
       </c>
     </row>
-    <row r="145" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A145" t="s">
         <v>9</v>
       </c>
@@ -10919,7 +10921,7 @@
         <v>15.268658439999999</v>
       </c>
     </row>
-    <row r="146" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A146" t="s">
         <v>9</v>
       </c>
@@ -10948,7 +10950,7 @@
         <v>15.304725729999999</v>
       </c>
     </row>
-    <row r="147" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A147" t="s">
         <v>9</v>
       </c>
@@ -10977,7 +10979,7 @@
         <v>15.29868785</v>
       </c>
     </row>
-    <row r="148" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A148" t="s">
         <v>9</v>
       </c>
@@ -11006,7 +11008,7 @@
         <v>15.24975221</v>
       </c>
     </row>
-    <row r="149" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A149" t="s">
         <v>9</v>
       </c>
@@ -11035,7 +11037,7 @@
         <v>15.22652497</v>
       </c>
     </row>
-    <row r="150" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A150" t="s">
         <v>9</v>
       </c>
@@ -11064,7 +11066,7 @@
         <v>17.16807189</v>
       </c>
     </row>
-    <row r="151" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A151" t="s">
         <v>9</v>
       </c>
@@ -11093,7 +11095,7 @@
         <v>15.19368246</v>
       </c>
     </row>
-    <row r="152" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A152" t="s">
         <v>9</v>
       </c>
@@ -11122,7 +11124,7 @@
         <v>15.377574210000001</v>
       </c>
     </row>
-    <row r="153" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A153" t="s">
         <v>9</v>
       </c>
@@ -11151,7 +11153,7 @@
         <v>15.582529040000001</v>
       </c>
     </row>
-    <row r="154" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A154" t="s">
         <v>9</v>
       </c>
@@ -11180,7 +11182,7 @@
         <v>20.814641949999999</v>
       </c>
     </row>
-    <row r="155" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A155" t="s">
         <v>9</v>
       </c>
@@ -11209,7 +11211,7 @@
         <v>20.548084150000001</v>
       </c>
     </row>
-    <row r="156" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A156" t="s">
         <v>9</v>
       </c>
@@ -11238,7 +11240,7 @@
         <v>15.40659252</v>
       </c>
     </row>
-    <row r="157" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A157" t="s">
         <v>9</v>
       </c>
@@ -11267,7 +11269,7 @@
         <v>15.369573279999999</v>
       </c>
     </row>
-    <row r="158" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A158" t="s">
         <v>9</v>
       </c>
@@ -11296,7 +11298,7 @@
         <v>19.39792302</v>
       </c>
     </row>
-    <row r="159" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A159" t="s">
         <v>9</v>
       </c>
@@ -11325,7 +11327,7 @@
         <v>18.951001720000001</v>
       </c>
     </row>
-    <row r="160" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A160" t="s">
         <v>9</v>
       </c>
@@ -11354,7 +11356,7 @@
         <v>20.74396715</v>
       </c>
     </row>
-    <row r="161" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A161" t="s">
         <v>9</v>
       </c>
@@ -11383,7 +11385,7 @@
         <v>19.401163180000001</v>
       </c>
     </row>
-    <row r="162" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A162" t="s">
         <v>9</v>
       </c>
@@ -11412,7 +11414,7 @@
         <v>19.767295149999999</v>
       </c>
     </row>
-    <row r="163" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A163" t="s">
         <v>9</v>
       </c>
@@ -11441,7 +11443,7 @@
         <v>19.703949359999999</v>
       </c>
     </row>
-    <row r="164" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A164" t="s">
         <v>9</v>
       </c>
@@ -11470,7 +11472,7 @@
         <v>20.41277929</v>
       </c>
     </row>
-    <row r="165" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A165" t="s">
         <v>9</v>
       </c>
@@ -11499,7 +11501,7 @@
         <v>22.17447125</v>
       </c>
     </row>
-    <row r="166" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A166" t="s">
         <v>9</v>
       </c>
@@ -11528,7 +11530,7 @@
         <v>21.195845720000001</v>
       </c>
     </row>
-    <row r="167" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A167" t="s">
         <v>9</v>
       </c>
@@ -11557,7 +11559,7 @@
         <v>20.40564393</v>
       </c>
     </row>
-    <row r="168" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="168" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A168" t="s">
         <v>9</v>
       </c>
@@ -11586,7 +11588,7 @@
         <v>20.084716159999999</v>
       </c>
     </row>
-    <row r="169" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="169" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A169" t="s">
         <v>9</v>
       </c>
@@ -11615,7 +11617,7 @@
         <v>19.843438070000001</v>
       </c>
     </row>
-    <row r="170" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="170" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A170" t="s">
         <v>9</v>
       </c>
@@ -11644,7 +11646,7 @@
         <v>20.369494230000001</v>
       </c>
     </row>
-    <row r="171" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="171" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A171" t="s">
         <v>9</v>
       </c>
@@ -11673,7 +11675,7 @@
         <v>20.032193029999998</v>
       </c>
     </row>
-    <row r="172" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="172" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A172" t="s">
         <v>9</v>
       </c>
@@ -11702,7 +11704,7 @@
         <v>19.53329149</v>
       </c>
     </row>
-    <row r="173" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="173" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A173" t="s">
         <v>9</v>
       </c>
@@ -11731,7 +11733,7 @@
         <v>25.659637400000001</v>
       </c>
     </row>
-    <row r="174" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="174" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A174" t="s">
         <v>9</v>
       </c>
@@ -11760,7 +11762,7 @@
         <v>25.88074611</v>
       </c>
     </row>
-    <row r="175" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A175" t="s">
         <v>9</v>
       </c>
@@ -11789,7 +11791,7 @@
         <v>25.960610280000001</v>
       </c>
     </row>
-    <row r="176" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="176" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A176" t="s">
         <v>9</v>
       </c>
@@ -11818,7 +11820,7 @@
         <v>15.28739519</v>
       </c>
     </row>
-    <row r="177" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="177" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A177" t="s">
         <v>9</v>
       </c>
@@ -11847,7 +11849,7 @@
         <v>15.300864219999999</v>
       </c>
     </row>
-    <row r="178" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="178" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A178" t="s">
         <v>9</v>
       </c>
@@ -11876,7 +11878,7 @@
         <v>25.229720270000001</v>
       </c>
     </row>
-    <row r="179" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="179" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A179" t="s">
         <v>9</v>
       </c>
@@ -11905,7 +11907,7 @@
         <v>25.09751314</v>
       </c>
     </row>
-    <row r="180" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="180" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A180" t="s">
         <v>9</v>
       </c>
@@ -11934,7 +11936,7 @@
         <v>25.402589429999999</v>
       </c>
     </row>
-    <row r="181" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A181" t="s">
         <v>9</v>
       </c>
@@ -11963,7 +11965,7 @@
         <v>25.292387000000002</v>
       </c>
     </row>
-    <row r="182" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A182" t="s">
         <v>9</v>
       </c>
@@ -11992,7 +11994,7 @@
         <v>24.156764710000001</v>
       </c>
     </row>
-    <row r="183" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="183" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A183" t="s">
         <v>9</v>
       </c>
@@ -12021,7 +12023,7 @@
         <v>28.868002659999998</v>
       </c>
     </row>
-    <row r="184" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A184" t="s">
         <v>9</v>
       </c>
@@ -12050,7 +12052,7 @@
         <v>29.109441520000001</v>
       </c>
     </row>
-    <row r="185" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="185" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A185" t="s">
         <v>9</v>
       </c>
@@ -12079,7 +12081,7 @@
         <v>26.367934210000001</v>
       </c>
     </row>
-    <row r="186" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="186" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A186" t="s">
         <v>9</v>
       </c>
@@ -12108,7 +12110,7 @@
         <v>26.33396948</v>
       </c>
     </row>
-    <row r="187" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="187" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A187" t="s">
         <v>9</v>
       </c>
@@ -12137,7 +12139,7 @@
         <v>24.50002233</v>
       </c>
     </row>
-    <row r="188" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="188" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A188" t="s">
         <v>9</v>
       </c>
@@ -12166,7 +12168,7 @@
         <v>28.15502798</v>
       </c>
     </row>
-    <row r="189" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="189" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A189" t="s">
         <v>9</v>
       </c>
@@ -12195,7 +12197,7 @@
         <v>27.39369434</v>
       </c>
     </row>
-    <row r="190" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A190" t="s">
         <v>9</v>
       </c>
@@ -12224,7 +12226,7 @@
         <v>26.323014910000001</v>
       </c>
     </row>
-    <row r="191" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="191" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A191" t="s">
         <v>9</v>
       </c>
@@ -12253,7 +12255,7 @@
         <v>26.75922675</v>
       </c>
     </row>
-    <row r="192" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="192" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A192" t="s">
         <v>9</v>
       </c>
@@ -12282,7 +12284,7 @@
         <v>26.282595560000001</v>
       </c>
     </row>
-    <row r="193" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="193" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A193" t="s">
         <v>9</v>
       </c>
@@ -12311,7 +12313,7 @@
         <v>27.388931719999999</v>
       </c>
     </row>
-    <row r="194" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="194" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A194" t="s">
         <v>9</v>
       </c>
@@ -12340,7 +12342,7 @@
         <v>26.48160356</v>
       </c>
     </row>
-    <row r="195" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="195" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A195" t="s">
         <v>9</v>
       </c>
@@ -12369,7 +12371,7 @@
         <v>29.027490660000002</v>
       </c>
     </row>
-    <row r="196" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="196" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A196" t="s">
         <v>9</v>
       </c>
@@ -12398,7 +12400,7 @@
         <v>27.934716420000001</v>
       </c>
     </row>
-    <row r="197" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="197" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A197" t="s">
         <v>9</v>
       </c>
@@ -12427,7 +12429,7 @@
         <v>28.073527370000001</v>
       </c>
     </row>
-    <row r="198" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="198" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A198" t="s">
         <v>9</v>
       </c>
@@ -12456,7 +12458,7 @@
         <v>26.603978359999999</v>
       </c>
     </row>
-    <row r="199" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="199" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A199" t="s">
         <v>9</v>
       </c>
@@ -12485,7 +12487,7 @@
         <v>26.649803070000001</v>
       </c>
     </row>
-    <row r="200" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="200" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A200" t="s">
         <v>9</v>
       </c>
@@ -12514,7 +12516,7 @@
         <v>23.47321444</v>
       </c>
     </row>
-    <row r="201" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="201" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A201" t="s">
         <v>9</v>
       </c>
@@ -12543,7 +12545,7 @@
         <v>23.755399319999999</v>
       </c>
     </row>
-    <row r="202" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="202" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A202" t="s">
         <v>9</v>
       </c>
@@ -12572,7 +12574,7 @@
         <v>23.211100779999999</v>
       </c>
     </row>
-    <row r="203" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="203" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A203" t="s">
         <v>9</v>
       </c>
@@ -12601,7 +12603,7 @@
         <v>22.763112679999999</v>
       </c>
     </row>
-    <row r="204" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="204" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A204" t="s">
         <v>9</v>
       </c>
@@ -12630,7 +12632,7 @@
         <v>22.146161379999999</v>
       </c>
     </row>
-    <row r="205" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="205" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A205" t="s">
         <v>9</v>
       </c>
@@ -12659,7 +12661,7 @@
         <v>22.336933590000001</v>
       </c>
     </row>
-    <row r="206" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="206" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A206" t="s">
         <v>9</v>
       </c>
@@ -12688,7 +12690,7 @@
         <v>22.092762520000001</v>
       </c>
     </row>
-    <row r="207" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="207" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A207" t="s">
         <v>9</v>
       </c>
@@ -12717,7 +12719,7 @@
         <v>22.038607559999999</v>
       </c>
     </row>
-    <row r="208" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="208" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A208" t="s">
         <v>9</v>
       </c>
@@ -12746,7 +12748,7 @@
         <v>22.703247279999999</v>
       </c>
     </row>
-    <row r="209" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="209" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A209" t="s">
         <v>9</v>
       </c>
@@ -12775,7 +12777,7 @@
         <v>22.89095331</v>
       </c>
     </row>
-    <row r="210" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="210" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A210" t="s">
         <v>9</v>
       </c>
@@ -12804,7 +12806,7 @@
         <v>22.676744920000001</v>
       </c>
     </row>
-    <row r="211" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="211" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A211" t="s">
         <v>9</v>
       </c>
@@ -12833,7 +12835,7 @@
         <v>27.333502979999999</v>
       </c>
     </row>
-    <row r="212" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="212" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A212" t="s">
         <v>9</v>
       </c>
@@ -12862,7 +12864,7 @@
         <v>26.59624668</v>
       </c>
     </row>
-    <row r="213" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="213" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A213" t="s">
         <v>9</v>
       </c>
@@ -12891,7 +12893,7 @@
         <v>25.592646439999999</v>
       </c>
     </row>
-    <row r="214" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="214" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A214" t="s">
         <v>9</v>
       </c>
@@ -12920,7 +12922,7 @@
         <v>25.956129099999998</v>
       </c>
     </row>
-    <row r="215" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="215" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A215" t="s">
         <v>9</v>
       </c>
@@ -12949,7 +12951,7 @@
         <v>26.916411920000002</v>
       </c>
     </row>
-    <row r="216" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="216" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A216" t="s">
         <v>9</v>
       </c>
@@ -12978,7 +12980,7 @@
         <v>17.358283289999999</v>
       </c>
     </row>
-    <row r="217" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="217" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A217" t="s">
         <v>9</v>
       </c>
@@ -13007,7 +13009,7 @@
         <v>16.909448780000002</v>
       </c>
     </row>
-    <row r="218" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="218" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A218" t="s">
         <v>9</v>
       </c>
@@ -13036,7 +13038,7 @@
         <v>16.579293910000001</v>
       </c>
     </row>
-    <row r="219" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="219" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A219" t="s">
         <v>9</v>
       </c>
@@ -13065,7 +13067,7 @@
         <v>16.03836557</v>
       </c>
     </row>
-    <row r="220" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="220" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A220" t="s">
         <v>9</v>
       </c>
@@ -13094,7 +13096,7 @@
         <v>16.156429379999999</v>
       </c>
     </row>
-    <row r="221" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="221" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A221" t="s">
         <v>9</v>
       </c>
@@ -13123,7 +13125,7 @@
         <v>14.308184649999999</v>
       </c>
     </row>
-    <row r="222" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="222" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A222" t="s">
         <v>9</v>
       </c>
@@ -13152,7 +13154,7 @@
         <v>13.88357961</v>
       </c>
     </row>
-    <row r="223" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="223" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A223" t="s">
         <v>9</v>
       </c>
@@ -13181,7 +13183,7 @@
         <v>12.828991650000001</v>
       </c>
     </row>
-    <row r="224" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="224" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A224" t="s">
         <v>9</v>
       </c>
@@ -13210,7 +13212,7 @@
         <v>12.693821209999999</v>
       </c>
     </row>
-    <row r="225" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="225" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A225" t="s">
         <v>9</v>
       </c>
@@ -13239,7 +13241,7 @@
         <v>13.174209490000001</v>
       </c>
     </row>
-    <row r="226" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="226" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A226" t="s">
         <v>9</v>
       </c>
@@ -13268,7 +13270,7 @@
         <v>14.25256882</v>
       </c>
     </row>
-    <row r="227" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="227" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A227" t="s">
         <v>9</v>
       </c>
@@ -13297,7 +13299,7 @@
         <v>14.654842370000001</v>
       </c>
     </row>
-    <row r="228" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="228" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A228" t="s">
         <v>9</v>
       </c>
@@ -13326,7 +13328,7 @@
         <v>15.144024529999999</v>
       </c>
     </row>
-    <row r="229" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="229" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A229" t="s">
         <v>9</v>
       </c>
@@ -13355,7 +13357,7 @@
         <v>18.569640360000001</v>
       </c>
     </row>
-    <row r="230" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="230" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A230" t="s">
         <v>9</v>
       </c>
@@ -13384,7 +13386,7 @@
         <v>18.830516920000001</v>
       </c>
     </row>
-    <row r="231" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="231" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A231" t="s">
         <v>9</v>
       </c>
@@ -13413,7 +13415,7 @@
         <v>18.69829043</v>
       </c>
     </row>
-    <row r="232" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="232" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A232" t="s">
         <v>9</v>
       </c>
@@ -13442,7 +13444,7 @@
         <v>19.044230769999999</v>
       </c>
     </row>
-    <row r="233" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="233" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A233" t="s">
         <v>9</v>
       </c>
@@ -13471,7 +13473,7 @@
         <v>19.718103540000001</v>
       </c>
     </row>
-    <row r="234" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="234" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A234" t="s">
         <v>9</v>
       </c>
@@ -13500,7 +13502,7 @@
         <v>20.876548809999999</v>
       </c>
     </row>
-    <row r="235" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="235" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A235" t="s">
         <v>9</v>
       </c>
@@ -13529,7 +13531,7 @@
         <v>21.03138358</v>
       </c>
     </row>
-    <row r="236" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="236" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A236" t="s">
         <v>9</v>
       </c>
@@ -13558,7 +13560,7 @@
         <v>22.204702269999999</v>
       </c>
     </row>
-    <row r="237" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="237" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A237" t="s">
         <v>9</v>
       </c>
@@ -13587,7 +13589,7 @@
         <v>23.028029780000001</v>
       </c>
     </row>
-    <row r="238" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="238" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A238" t="s">
         <v>9</v>
       </c>
@@ -13616,7 +13618,7 @@
         <v>23.73425202</v>
       </c>
     </row>
-    <row r="239" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="239" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A239" t="s">
         <v>9</v>
       </c>
@@ -13645,7 +13647,7 @@
         <v>24.642286429999999</v>
       </c>
     </row>
-    <row r="240" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="240" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A240" t="s">
         <v>9</v>
       </c>
@@ -13674,7 +13676,7 @@
         <v>26.07259981</v>
       </c>
     </row>
-    <row r="241" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="241" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A241" t="s">
         <v>9</v>
       </c>
@@ -13703,7 +13705,7 @@
         <v>24.238614649999999</v>
       </c>
     </row>
-    <row r="242" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="242" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A242" t="s">
         <v>9</v>
       </c>
@@ -13732,7 +13734,7 @@
         <v>19.259778090000001</v>
       </c>
     </row>
-    <row r="243" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="243" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A243" t="s">
         <v>9</v>
       </c>
@@ -13761,7 +13763,7 @@
         <v>19.25779245</v>
       </c>
     </row>
-    <row r="244" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="244" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A244" t="s">
         <v>9</v>
       </c>
@@ -13790,7 +13792,7 @@
         <v>20.084859959999999</v>
       </c>
     </row>
-    <row r="245" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="245" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A245" t="s">
         <v>9</v>
       </c>
@@ -13819,7 +13821,7 @@
         <v>19.899820630000001</v>
       </c>
     </row>
-    <row r="246" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="246" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A246" t="s">
         <v>9</v>
       </c>
@@ -13848,7 +13850,7 @@
         <v>27.29038259</v>
       </c>
     </row>
-    <row r="247" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="247" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A247" t="s">
         <v>9</v>
       </c>
@@ -13877,7 +13879,7 @@
         <v>26.558661019999999</v>
       </c>
     </row>
-    <row r="248" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="248" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A248" t="s">
         <v>9</v>
       </c>
@@ -13906,7 +13908,7 @@
         <v>26.891946090000001</v>
       </c>
     </row>
-    <row r="249" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="249" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A249" t="s">
         <v>9</v>
       </c>
@@ -13935,7 +13937,7 @@
         <v>25.95965086</v>
       </c>
     </row>
-    <row r="250" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="250" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A250" t="s">
         <v>9</v>
       </c>
@@ -13964,7 +13966,7 @@
         <v>25.96660078</v>
       </c>
     </row>
-    <row r="251" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="251" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A251" t="s">
         <v>9</v>
       </c>
@@ -13993,7 +13995,7 @@
         <v>25.811074130000002</v>
       </c>
     </row>
-    <row r="252" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="252" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A252" t="s">
         <v>9</v>
       </c>
@@ -14022,7 +14024,7 @@
         <v>25.135635019999999</v>
       </c>
     </row>
-    <row r="253" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="253" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A253" t="s">
         <v>9</v>
       </c>
@@ -14051,7 +14053,7 @@
         <v>25.107443809999999</v>
       </c>
     </row>
-    <row r="254" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="254" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A254" t="s">
         <v>9</v>
       </c>
@@ -14080,7 +14082,7 @@
         <v>25.716675469999998</v>
       </c>
     </row>
-    <row r="255" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="255" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A255" t="s">
         <v>9</v>
       </c>
@@ -14109,7 +14111,7 @@
         <v>26.63407729</v>
       </c>
     </row>
-    <row r="256" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="256" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A256" t="s">
         <v>9</v>
       </c>
@@ -14138,7 +14140,7 @@
         <v>27.268394000000001</v>
       </c>
     </row>
-    <row r="257" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="257" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A257" t="s">
         <v>9</v>
       </c>
@@ -14167,7 +14169,7 @@
         <v>26.685943129999998</v>
       </c>
     </row>
-    <row r="258" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="258" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A258" t="s">
         <v>9</v>
       </c>
@@ -14196,7 +14198,7 @@
         <v>27.142364749999999</v>
       </c>
     </row>
-    <row r="259" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="259" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A259" t="s">
         <v>9</v>
       </c>
@@ -14225,7 +14227,7 @@
         <v>26.508603170000001</v>
       </c>
     </row>
-    <row r="260" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="260" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A260" t="s">
         <v>9</v>
       </c>
@@ -14254,7 +14256,7 @@
         <v>24.888465669999999</v>
       </c>
     </row>
-    <row r="261" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="261" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A261" t="s">
         <v>9</v>
       </c>
@@ -14283,7 +14285,7 @@
         <v>25.22503983</v>
       </c>
     </row>
-    <row r="262" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="262" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A262" t="s">
         <v>9</v>
       </c>
@@ -14312,7 +14314,7 @@
         <v>18.809469409999998</v>
       </c>
     </row>
-    <row r="263" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="263" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A263" t="s">
         <v>9</v>
       </c>
@@ -14341,7 +14343,7 @@
         <v>27.775720710000002</v>
       </c>
     </row>
-    <row r="264" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="264" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A264" t="s">
         <v>9</v>
       </c>
@@ -14370,7 +14372,7 @@
         <v>27.708254969999999</v>
       </c>
     </row>
-    <row r="265" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="265" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A265" t="s">
         <v>9</v>
       </c>
@@ -14399,7 +14401,7 @@
         <v>27.61357143</v>
       </c>
     </row>
-    <row r="266" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="266" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A266" t="s">
         <v>9</v>
       </c>
@@ -14428,7 +14430,7 @@
         <v>29.006691050000001</v>
       </c>
     </row>
-    <row r="267" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="267" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A267" t="s">
         <v>9</v>
       </c>
@@ -14457,7 +14459,7 @@
         <v>27.6742235</v>
       </c>
     </row>
-    <row r="268" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="268" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A268" t="s">
         <v>9</v>
       </c>
@@ -14486,7 +14488,7 @@
         <v>27.058831739999999</v>
       </c>
     </row>
-    <row r="269" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="269" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A269" t="s">
         <v>9</v>
       </c>
@@ -14515,7 +14517,7 @@
         <v>28.198437800000001</v>
       </c>
     </row>
-    <row r="270" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="270" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A270" t="s">
         <v>9</v>
       </c>
@@ -14544,7 +14546,7 @@
         <v>27.088321530000002</v>
       </c>
     </row>
-    <row r="271" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="271" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A271" t="s">
         <v>9</v>
       </c>
@@ -14573,7 +14575,7 @@
         <v>26.689913199999999</v>
       </c>
     </row>
-    <row r="272" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="272" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A272" t="s">
         <v>9</v>
       </c>
@@ -14602,7 +14604,7 @@
         <v>28.22580044</v>
       </c>
     </row>
-    <row r="273" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="273" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A273" t="s">
         <v>9</v>
       </c>
@@ -14631,7 +14633,7 @@
         <v>27.863198700000002</v>
       </c>
     </row>
-    <row r="274" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="274" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A274" t="s">
         <v>9</v>
       </c>
@@ -14660,7 +14662,7 @@
         <v>27.925110190000002</v>
       </c>
     </row>
-    <row r="275" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="275" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A275" t="s">
         <v>9</v>
       </c>
@@ -14689,7 +14691,7 @@
         <v>22.808085269999999</v>
       </c>
     </row>
-    <row r="276" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="276" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A276" t="s">
         <v>9</v>
       </c>
@@ -14718,7 +14720,7 @@
         <v>22.974143059999999</v>
       </c>
     </row>
-    <row r="277" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="277" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A277" t="s">
         <v>9</v>
       </c>
@@ -14747,7 +14749,7 @@
         <v>20.740523119999999</v>
       </c>
     </row>
-    <row r="278" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="278" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A278" t="s">
         <v>9</v>
       </c>
@@ -14776,7 +14778,7 @@
         <v>21.489491350000002</v>
       </c>
     </row>
-    <row r="279" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="279" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A279" t="s">
         <v>9</v>
       </c>
@@ -14805,7 +14807,7 @@
         <v>22.09550827</v>
       </c>
     </row>
-    <row r="280" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="280" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A280" t="s">
         <v>9</v>
       </c>
@@ -14834,7 +14836,7 @@
         <v>22.692723010000002</v>
       </c>
     </row>
-    <row r="281" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="281" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A281" t="s">
         <v>9</v>
       </c>
@@ -14863,7 +14865,7 @@
         <v>22.757806080000002</v>
       </c>
     </row>
-    <row r="282" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="282" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A282" t="s">
         <v>9</v>
       </c>
@@ -14892,7 +14894,7 @@
         <v>22.97061321</v>
       </c>
     </row>
-    <row r="283" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="283" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A283" t="s">
         <v>9</v>
       </c>
@@ -14921,7 +14923,7 @@
         <v>21.6743591</v>
       </c>
     </row>
-    <row r="284" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="284" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A284" t="s">
         <v>9</v>
       </c>
@@ -14950,7 +14952,7 @@
         <v>21.999188419999999</v>
       </c>
     </row>
-    <row r="285" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="285" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A285" t="s">
         <v>9</v>
       </c>
@@ -14979,7 +14981,7 @@
         <v>21.227856150000001</v>
       </c>
     </row>
-    <row r="286" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="286" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A286" t="s">
         <v>9</v>
       </c>
@@ -15008,7 +15010,7 @@
         <v>21.754848450000001</v>
       </c>
     </row>
-    <row r="287" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="287" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A287" t="s">
         <v>9</v>
       </c>
@@ -15037,7 +15039,7 @@
         <v>22.513107380000001</v>
       </c>
     </row>
-    <row r="288" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="288" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A288" t="s">
         <v>9</v>
       </c>
@@ -15066,7 +15068,7 @@
         <v>22.49382563</v>
       </c>
     </row>
-    <row r="289" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="289" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A289" t="s">
         <v>9</v>
       </c>
@@ -15095,7 +15097,7 @@
         <v>22.330866019999998</v>
       </c>
     </row>
-    <row r="290" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="290" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A290" t="s">
         <v>9</v>
       </c>
@@ -15124,7 +15126,7 @@
         <v>22.404764010000001</v>
       </c>
     </row>
-    <row r="291" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="291" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A291" t="s">
         <v>9</v>
       </c>
@@ -15153,7 +15155,7 @@
         <v>22.466819820000001</v>
       </c>
     </row>
-    <row r="292" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="292" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A292" t="s">
         <v>9</v>
       </c>
@@ -15182,7 +15184,7 @@
         <v>22.266146880000001</v>
       </c>
     </row>
-    <row r="293" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="293" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A293" t="s">
         <v>9</v>
       </c>
@@ -15211,7 +15213,7 @@
         <v>21.866212910000002</v>
       </c>
     </row>
-    <row r="294" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="294" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A294" t="s">
         <v>9</v>
       </c>
@@ -15240,7 +15242,7 @@
         <v>22.58268009</v>
       </c>
     </row>
-    <row r="295" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="295" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A295" t="s">
         <v>9</v>
       </c>
@@ -15269,7 +15271,7 @@
         <v>22.113587039999999</v>
       </c>
     </row>
-    <row r="296" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="296" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A296" t="s">
         <v>9</v>
       </c>
@@ -15298,7 +15300,7 @@
         <v>22.061622679999999</v>
       </c>
     </row>
-    <row r="297" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="297" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A297" t="s">
         <v>9</v>
       </c>
@@ -15327,7 +15329,7 @@
         <v>22.920219419999999</v>
       </c>
     </row>
-    <row r="298" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="298" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A298" t="s">
         <v>9</v>
       </c>
@@ -15356,7 +15358,7 @@
         <v>21.073639660000001</v>
       </c>
     </row>
-    <row r="299" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="299" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A299" t="s">
         <v>9</v>
       </c>
@@ -15385,7 +15387,7 @@
         <v>22.7983364</v>
       </c>
     </row>
-    <row r="300" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="300" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A300" t="s">
         <v>9</v>
       </c>
@@ -15414,7 +15416,7 @@
         <v>22.151037110000001</v>
       </c>
     </row>
-    <row r="301" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="301" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A301" t="s">
         <v>9</v>
       </c>
@@ -15443,7 +15445,7 @@
         <v>30.110211719999999</v>
       </c>
     </row>
-    <row r="302" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="302" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A302" t="s">
         <v>9</v>
       </c>
@@ -15472,7 +15474,7 @@
         <v>30.223441950000002</v>
       </c>
     </row>
-    <row r="303" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="303" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A303" t="s">
         <v>9</v>
       </c>
@@ -15501,7 +15503,7 @@
         <v>30.789773</v>
       </c>
     </row>
-    <row r="304" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="304" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A304" t="s">
         <v>9</v>
       </c>
@@ -15530,7 +15532,7 @@
         <v>30.826683920000001</v>
       </c>
     </row>
-    <row r="305" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="305" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A305" t="s">
         <v>9</v>
       </c>
@@ -15559,7 +15561,7 @@
         <v>30.410237930000001</v>
       </c>
     </row>
-    <row r="306" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="306" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A306" t="s">
         <v>9</v>
       </c>
@@ -15588,7 +15590,7 @@
         <v>30.177986570000002</v>
       </c>
     </row>
-    <row r="307" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="307" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A307" t="s">
         <v>9</v>
       </c>
@@ -15617,7 +15619,7 @@
         <v>30.55534398</v>
       </c>
     </row>
-    <row r="308" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="308" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A308" t="s">
         <v>9</v>
       </c>
@@ -15646,7 +15648,7 @@
         <v>30.548688739999999</v>
       </c>
     </row>
-    <row r="309" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="309" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A309" t="s">
         <v>9</v>
       </c>
@@ -15675,7 +15677,7 @@
         <v>30.595714999999998</v>
       </c>
     </row>
-    <row r="310" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="310" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A310" t="s">
         <v>9</v>
       </c>
@@ -15704,7 +15706,7 @@
         <v>30.741103620000001</v>
       </c>
     </row>
-    <row r="311" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="311" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A311" t="s">
         <v>9</v>
       </c>
@@ -15733,7 +15735,7 @@
         <v>29.94440174</v>
       </c>
     </row>
-    <row r="312" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="312" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A312" t="s">
         <v>9</v>
       </c>
@@ -15762,7 +15764,7 @@
         <v>30.324742929999999</v>
       </c>
     </row>
-    <row r="313" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="313" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A313" t="s">
         <v>9</v>
       </c>
@@ -15791,7 +15793,7 @@
         <v>30.220459330000001</v>
       </c>
     </row>
-    <row r="314" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="314" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A314" t="s">
         <v>9</v>
       </c>
@@ -15820,7 +15822,7 @@
         <v>30.08494061</v>
       </c>
     </row>
-    <row r="315" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="315" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A315" t="s">
         <v>9</v>
       </c>
@@ -15849,7 +15851,7 @@
         <v>29.915665239999999</v>
       </c>
     </row>
-    <row r="316" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="316" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A316" t="s">
         <v>9</v>
       </c>
@@ -15878,7 +15880,7 @@
         <v>29.643007520000001</v>
       </c>
     </row>
-    <row r="317" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="317" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A317" t="s">
         <v>9</v>
       </c>
@@ -15907,7 +15909,7 @@
         <v>30.23249719</v>
       </c>
     </row>
-    <row r="318" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="318" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A318" t="s">
         <v>9</v>
       </c>
@@ -15936,7 +15938,7 @@
         <v>30.002984829999999</v>
       </c>
     </row>
-    <row r="319" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="319" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A319" t="s">
         <v>9</v>
       </c>
@@ -15965,7 +15967,7 @@
         <v>27.979859860000001</v>
       </c>
     </row>
-    <row r="320" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="320" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A320" t="s">
         <v>9</v>
       </c>
@@ -15994,7 +15996,7 @@
         <v>29.193835830000001</v>
       </c>
     </row>
-    <row r="321" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="321" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A321" t="s">
         <v>9</v>
       </c>
@@ -16023,7 +16025,7 @@
         <v>29.441858920000001</v>
       </c>
     </row>
-    <row r="322" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="322" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A322" t="s">
         <v>9</v>
       </c>
@@ -16052,7 +16054,7 @@
         <v>30.374914350000001</v>
       </c>
     </row>
-    <row r="323" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="323" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A323" t="s">
         <v>9</v>
       </c>
@@ -16081,7 +16083,7 @@
         <v>27.758114760000002</v>
       </c>
     </row>
-    <row r="324" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="324" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A324" t="s">
         <v>9</v>
       </c>
@@ -16110,7 +16112,7 @@
         <v>27.296590330000001</v>
       </c>
     </row>
-    <row r="325" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="325" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A325" t="s">
         <v>9</v>
       </c>
@@ -16139,7 +16141,7 @@
         <v>27.911669969999998</v>
       </c>
     </row>
-    <row r="326" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="326" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A326" t="s">
         <v>9</v>
       </c>
@@ -16168,7 +16170,7 @@
         <v>27.668624009999998</v>
       </c>
     </row>
-    <row r="327" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="327" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A327" t="s">
         <v>9</v>
       </c>
@@ -16197,7 +16199,7 @@
         <v>27.587541940000001</v>
       </c>
     </row>
-    <row r="328" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="328" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A328" t="s">
         <v>9</v>
       </c>
@@ -16226,7 +16228,7 @@
         <v>27.901685969999999</v>
       </c>
     </row>
-    <row r="329" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="329" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A329" t="s">
         <v>9</v>
       </c>
@@ -16255,7 +16257,7 @@
         <v>27.964169120000001</v>
       </c>
     </row>
-    <row r="330" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="330" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A330" t="s">
         <v>9</v>
       </c>
@@ -16284,7 +16286,7 @@
         <v>28.69974401</v>
       </c>
     </row>
-    <row r="331" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="331" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A331" t="s">
         <v>9</v>
       </c>
@@ -16313,7 +16315,7 @@
         <v>30.755949170000001</v>
       </c>
     </row>
-    <row r="332" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="332" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A332" t="s">
         <v>9</v>
       </c>
@@ -16342,7 +16344,7 @@
         <v>30.918677599999999</v>
       </c>
     </row>
-    <row r="333" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="333" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A333" t="s">
         <v>9</v>
       </c>
@@ -16371,7 +16373,7 @@
         <v>31.061257099999999</v>
       </c>
     </row>
-    <row r="334" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="334" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A334" t="s">
         <v>9</v>
       </c>
@@ -16400,7 +16402,7 @@
         <v>31.154728349999999</v>
       </c>
     </row>
-    <row r="335" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="335" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A335" t="s">
         <v>9</v>
       </c>
@@ -16429,7 +16431,7 @@
         <v>30.94170506</v>
       </c>
     </row>
-    <row r="336" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="336" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A336" t="s">
         <v>9</v>
       </c>
@@ -16458,7 +16460,7 @@
         <v>30.00666416</v>
       </c>
     </row>
-    <row r="337" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="337" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A337" t="s">
         <v>9</v>
       </c>
@@ -16487,7 +16489,7 @@
         <v>30.481006860000001</v>
       </c>
     </row>
-    <row r="338" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="338" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A338" t="s">
         <v>9</v>
       </c>
@@ -16516,7 +16518,7 @@
         <v>30.343667620000002</v>
       </c>
     </row>
-    <row r="339" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="339" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A339" t="s">
         <v>9</v>
       </c>
@@ -16545,7 +16547,7 @@
         <v>30.50611533</v>
       </c>
     </row>
-    <row r="340" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="340" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A340" t="s">
         <v>9</v>
       </c>
@@ -16574,7 +16576,7 @@
         <v>30.736491919999999</v>
       </c>
     </row>
-    <row r="341" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="341" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A341" t="s">
         <v>9</v>
       </c>
@@ -16603,7 +16605,7 @@
         <v>30.733002339999999</v>
       </c>
     </row>
-    <row r="342" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="342" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A342" t="s">
         <v>9</v>
       </c>
@@ -16632,7 +16634,7 @@
         <v>30.734852239999999</v>
       </c>
     </row>
-    <row r="343" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="343" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A343" t="s">
         <v>9</v>
       </c>
@@ -16661,7 +16663,7 @@
         <v>30.413161429999999</v>
       </c>
     </row>
-    <row r="344" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="344" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A344" t="s">
         <v>9</v>
       </c>
@@ -16690,7 +16692,7 @@
         <v>30.596640690000001</v>
       </c>
     </row>
-    <row r="345" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="345" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A345" t="s">
         <v>9</v>
       </c>
@@ -16719,7 +16721,7 @@
         <v>29.83208368</v>
       </c>
     </row>
-    <row r="346" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="346" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A346" t="s">
         <v>9</v>
       </c>
@@ -16748,7 +16750,7 @@
         <v>28.9905866</v>
       </c>
     </row>
-    <row r="347" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="347" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A347" t="s">
         <v>9</v>
       </c>
@@ -16777,7 +16779,7 @@
         <v>28.994870410000001</v>
       </c>
     </row>
-    <row r="348" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="348" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A348" t="s">
         <v>9</v>
       </c>
@@ -16806,7 +16808,7 @@
         <v>29.720894019999999</v>
       </c>
     </row>
-    <row r="349" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="349" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A349" t="s">
         <v>9</v>
       </c>
@@ -16835,7 +16837,7 @@
         <v>22.299687120000002</v>
       </c>
     </row>
-    <row r="350" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="350" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A350" t="s">
         <v>9</v>
       </c>
@@ -16864,7 +16866,7 @@
         <v>22.64118255</v>
       </c>
     </row>
-    <row r="351" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="351" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A351" t="s">
         <v>9</v>
       </c>
@@ -16893,7 +16895,7 @@
         <v>23.40009221</v>
       </c>
     </row>
-    <row r="352" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="352" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A352" t="s">
         <v>9</v>
       </c>
@@ -16922,7 +16924,7 @@
         <v>22.432332049999999</v>
       </c>
     </row>
-    <row r="353" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="353" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A353" t="s">
         <v>9</v>
       </c>
@@ -16951,7 +16953,7 @@
         <v>15.78221216</v>
       </c>
     </row>
-    <row r="354" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="354" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A354" t="s">
         <v>9</v>
       </c>
@@ -16980,7 +16982,7 @@
         <v>15.623652229999999</v>
       </c>
     </row>
-    <row r="355" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="355" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A355" t="s">
         <v>9</v>
       </c>
@@ -17009,7 +17011,7 @@
         <v>23.83544251</v>
       </c>
     </row>
-    <row r="356" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="356" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A356" t="s">
         <v>9</v>
       </c>
@@ -17038,7 +17040,7 @@
         <v>17.83245251</v>
       </c>
     </row>
-    <row r="357" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="357" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A357" t="s">
         <v>9</v>
       </c>
@@ -17067,7 +17069,7 @@
         <v>16.380791760000001</v>
       </c>
     </row>
-    <row r="358" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="358" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A358" t="s">
         <v>9</v>
       </c>
@@ -17096,7 +17098,7 @@
         <v>17.182437960000001</v>
       </c>
     </row>
-    <row r="359" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="359" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A359" t="s">
         <v>9</v>
       </c>
@@ -17125,7 +17127,7 @@
         <v>16.67795812</v>
       </c>
     </row>
-    <row r="360" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="360" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A360" t="s">
         <v>9</v>
       </c>
@@ -17154,7 +17156,7 @@
         <v>19.017444609999998</v>
       </c>
     </row>
-    <row r="361" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="361" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A361" t="s">
         <v>9</v>
       </c>
@@ -17183,7 +17185,7 @@
         <v>19.007788640000001</v>
       </c>
     </row>
-    <row r="362" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="362" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A362" t="s">
         <v>9</v>
       </c>
@@ -17212,7 +17214,7 @@
         <v>22.46659704</v>
       </c>
     </row>
-    <row r="363" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="363" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A363" t="s">
         <v>9</v>
       </c>
@@ -17241,7 +17243,7 @@
         <v>25.135924159999998</v>
       </c>
     </row>
-    <row r="364" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="364" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A364" t="s">
         <v>9</v>
       </c>
@@ -17270,7 +17272,7 @@
         <v>19.849837279999999</v>
       </c>
     </row>
-    <row r="365" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="365" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A365" t="s">
         <v>9</v>
       </c>
@@ -17299,7 +17301,7 @@
         <v>21.40159027</v>
       </c>
     </row>
-    <row r="366" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="366" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A366" t="s">
         <v>9</v>
       </c>
@@ -17328,7 +17330,7 @@
         <v>18.954282890000002</v>
       </c>
     </row>
-    <row r="367" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="367" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A367" t="s">
         <v>9</v>
       </c>
@@ -17357,7 +17359,7 @@
         <v>21.238506610000002</v>
       </c>
     </row>
-    <row r="368" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="368" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A368" t="s">
         <v>9</v>
       </c>
@@ -17386,7 +17388,7 @@
         <v>20.707198290000001</v>
       </c>
     </row>
-    <row r="369" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="369" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A369" t="s">
         <v>9</v>
       </c>
@@ -17415,7 +17417,7 @@
         <v>17.78576696</v>
       </c>
     </row>
-    <row r="370" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="370" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A370" t="s">
         <v>9</v>
       </c>
@@ -17444,7 +17446,7 @@
         <v>15.357908200000001</v>
       </c>
     </row>
-    <row r="371" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="371" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A371" t="s">
         <v>9</v>
       </c>
@@ -17473,7 +17475,7 @@
         <v>23.753775000000001</v>
       </c>
     </row>
-    <row r="372" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="372" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A372" t="s">
         <v>9</v>
       </c>
@@ -17502,7 +17504,7 @@
         <v>23.143199800000001</v>
       </c>
     </row>
-    <row r="373" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="373" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A373" t="s">
         <v>9</v>
       </c>
@@ -17531,7 +17533,7 @@
         <v>23.466027</v>
       </c>
     </row>
-    <row r="374" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="374" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A374" t="s">
         <v>9</v>
       </c>
@@ -17560,7 +17562,7 @@
         <v>25.117663690000001</v>
       </c>
     </row>
-    <row r="375" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="375" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A375" t="s">
         <v>9</v>
       </c>
@@ -17589,7 +17591,7 @@
         <v>25.087773729999999</v>
       </c>
     </row>
-    <row r="376" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="376" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A376" t="s">
         <v>9</v>
       </c>
@@ -17618,7 +17620,7 @@
         <v>25.684785959999999</v>
       </c>
     </row>
-    <row r="377" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="377" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A377" t="s">
         <v>9</v>
       </c>
@@ -17647,7 +17649,7 @@
         <v>23.449682190000001</v>
       </c>
     </row>
-    <row r="378" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="378" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A378" t="s">
         <v>9</v>
       </c>
@@ -17676,7 +17678,7 @@
         <v>24.65141667</v>
       </c>
     </row>
-    <row r="379" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="379" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A379" t="s">
         <v>9</v>
       </c>
@@ -17705,7 +17707,7 @@
         <v>27.231989729999999</v>
       </c>
     </row>
-    <row r="380" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="380" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A380" t="s">
         <v>9</v>
       </c>
@@ -17734,7 +17736,7 @@
         <v>22.39079452</v>
       </c>
     </row>
-    <row r="381" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="381" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A381" t="s">
         <v>9</v>
       </c>
@@ -17763,7 +17765,7 @@
         <v>26.99670506</v>
       </c>
     </row>
-    <row r="382" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="382" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A382" t="s">
         <v>9</v>
       </c>
@@ -17792,7 +17794,7 @@
         <v>29.485896969999999</v>
       </c>
     </row>
-    <row r="383" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="383" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A383" t="s">
         <v>9</v>
       </c>
@@ -17821,7 +17823,7 @@
         <v>29.211454839999998</v>
       </c>
     </row>
-    <row r="384" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="384" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A384" t="s">
         <v>9</v>
       </c>
@@ -17850,7 +17852,7 @@
         <v>28.96787604</v>
       </c>
     </row>
-    <row r="385" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="385" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A385" t="s">
         <v>9</v>
       </c>
@@ -17879,7 +17881,7 @@
         <v>29.559462289999999</v>
       </c>
     </row>
-    <row r="386" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="386" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A386" t="s">
         <v>9</v>
       </c>
@@ -17908,7 +17910,7 @@
         <v>29.360647100000001</v>
       </c>
     </row>
-    <row r="387" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="387" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A387" t="s">
         <v>9</v>
       </c>
@@ -17937,7 +17939,7 @@
         <v>28.44505345</v>
       </c>
     </row>
-    <row r="388" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="388" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A388" t="s">
         <v>9</v>
       </c>
@@ -17966,7 +17968,7 @@
         <v>29.742382070000001</v>
       </c>
     </row>
-    <row r="389" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="389" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A389" t="s">
         <v>9</v>
       </c>
@@ -17995,7 +17997,7 @@
         <v>29.829629629999999</v>
       </c>
     </row>
-    <row r="390" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="390" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A390" t="s">
         <v>9</v>
       </c>
@@ -18024,7 +18026,7 @@
         <v>29.59941624</v>
       </c>
     </row>
-    <row r="391" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="391" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A391" t="s">
         <v>9</v>
       </c>
@@ -18053,7 +18055,7 @@
         <v>29.521794320000001</v>
       </c>
     </row>
-    <row r="392" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="392" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A392" t="s">
         <v>9</v>
       </c>
@@ -18082,7 +18084,7 @@
         <v>29.539442579999999</v>
       </c>
     </row>
-    <row r="393" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="393" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A393" t="s">
         <v>9</v>
       </c>
@@ -18111,7 +18113,7 @@
         <v>29.4007161</v>
       </c>
     </row>
-    <row r="394" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="394" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A394" t="s">
         <v>9</v>
       </c>
@@ -18140,7 +18142,7 @@
         <v>29.112979599999999</v>
       </c>
     </row>
-    <row r="395" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="395" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A395" t="s">
         <v>9</v>
       </c>
@@ -18169,7 +18171,7 @@
         <v>29.469530599999999</v>
       </c>
     </row>
-    <row r="396" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="396" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A396" t="s">
         <v>9</v>
       </c>
@@ -18198,7 +18200,7 @@
         <v>29.254109889999999</v>
       </c>
     </row>
-    <row r="397" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="397" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A397" t="s">
         <v>9</v>
       </c>
@@ -18227,7 +18229,7 @@
         <v>28.658989519999999</v>
       </c>
     </row>
-    <row r="398" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="398" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A398" t="s">
         <v>9</v>
       </c>
@@ -18256,7 +18258,7 @@
         <v>29.259908100000001</v>
       </c>
     </row>
-    <row r="399" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="399" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A399" t="s">
         <v>9</v>
       </c>
@@ -18285,7 +18287,7 @@
         <v>29.323707670000001</v>
       </c>
     </row>
-    <row r="400" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="400" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A400" t="s">
         <v>9</v>
       </c>
@@ -18314,7 +18316,7 @@
         <v>28.972676530000001</v>
       </c>
     </row>
-    <row r="401" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="401" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A401" t="s">
         <v>9</v>
       </c>
@@ -18343,7 +18345,7 @@
         <v>29.180208799999999</v>
       </c>
     </row>
-    <row r="402" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="402" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A402" t="s">
         <v>9</v>
       </c>
@@ -18372,7 +18374,7 @@
         <v>29.208925170000001</v>
       </c>
     </row>
-    <row r="403" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="403" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A403" t="s">
         <v>9</v>
       </c>
@@ -18401,7 +18403,7 @@
         <v>28.412674419999998</v>
       </c>
     </row>
-    <row r="404" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="404" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A404" t="s">
         <v>9</v>
       </c>
@@ -18430,7 +18432,7 @@
         <v>28.729656590000001</v>
       </c>
     </row>
-    <row r="405" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="405" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A405" t="s">
         <v>9</v>
       </c>
@@ -18459,7 +18461,7 @@
         <v>28.90291144</v>
       </c>
     </row>
-    <row r="406" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="406" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A406" t="s">
         <v>9</v>
       </c>
@@ -18488,7 +18490,7 @@
         <v>29.004626559999998</v>
       </c>
     </row>
-    <row r="407" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="407" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A407" t="s">
         <v>9</v>
       </c>
@@ -18517,7 +18519,7 @@
         <v>28.454836759999999</v>
       </c>
     </row>
-    <row r="408" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="408" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A408" t="s">
         <v>9</v>
       </c>
@@ -18546,7 +18548,7 @@
         <v>27.76395398</v>
       </c>
     </row>
-    <row r="409" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="409" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A409" t="s">
         <v>9</v>
       </c>
@@ -18575,7 +18577,7 @@
         <v>29.188519490000001</v>
       </c>
     </row>
-    <row r="410" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="410" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A410" t="s">
         <v>9</v>
       </c>
@@ -18604,7 +18606,7 @@
         <v>29.51489419</v>
       </c>
     </row>
-    <row r="411" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="411" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A411" t="s">
         <v>9</v>
       </c>
@@ -18633,7 +18635,7 @@
         <v>28.983547990000002</v>
       </c>
     </row>
-    <row r="412" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="412" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A412" t="s">
         <v>9</v>
       </c>
@@ -18662,7 +18664,7 @@
         <v>29.250630090000001</v>
       </c>
     </row>
-    <row r="413" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="413" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A413" t="s">
         <v>9</v>
       </c>
@@ -18691,7 +18693,7 @@
         <v>28.778369640000001</v>
       </c>
     </row>
-    <row r="414" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="414" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A414" t="s">
         <v>9</v>
       </c>
@@ -18720,7 +18722,7 @@
         <v>29.252790050000002</v>
       </c>
     </row>
-    <row r="415" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="415" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A415" t="s">
         <v>9</v>
       </c>
@@ -18749,7 +18751,7 @@
         <v>28.117313469999999</v>
       </c>
     </row>
-    <row r="416" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="416" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A416" t="s">
         <v>9</v>
       </c>
@@ -18778,7 +18780,7 @@
         <v>28.702237849999999</v>
       </c>
     </row>
-    <row r="417" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="417" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A417" t="s">
         <v>9</v>
       </c>
@@ -18807,7 +18809,7 @@
         <v>28.823505770000001</v>
       </c>
     </row>
-    <row r="418" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="418" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A418" t="s">
         <v>9</v>
       </c>
@@ -18836,7 +18838,7 @@
         <v>28.867088330000001</v>
       </c>
     </row>
-    <row r="419" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="419" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A419" t="s">
         <v>9</v>
       </c>
@@ -18865,7 +18867,7 @@
         <v>28.904640279999999</v>
       </c>
     </row>
-    <row r="420" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="420" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A420" t="s">
         <v>9</v>
       </c>
@@ -18894,7 +18896,7 @@
         <v>28.713670700000002</v>
       </c>
     </row>
-    <row r="421" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="421" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A421" t="s">
         <v>9</v>
       </c>
@@ -18923,7 +18925,7 @@
         <v>28.561151250000002</v>
       </c>
     </row>
-    <row r="422" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="422" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A422" t="s">
         <v>9</v>
       </c>
@@ -18952,7 +18954,7 @@
         <v>28.696449659999999</v>
       </c>
     </row>
-    <row r="423" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="423" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A423" t="s">
         <v>9</v>
       </c>
@@ -18981,7 +18983,7 @@
         <v>28.926836689999998</v>
       </c>
     </row>
-    <row r="424" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="424" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A424" t="s">
         <v>9</v>
       </c>
@@ -19010,7 +19012,7 @@
         <v>28.408641230000001</v>
       </c>
     </row>
-    <row r="425" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="425" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A425" t="s">
         <v>9</v>
       </c>
@@ -19039,7 +19041,7 @@
         <v>28.484755920000001</v>
       </c>
     </row>
-    <row r="426" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="426" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A426" t="s">
         <v>9</v>
       </c>
@@ -19068,7 +19070,7 @@
         <v>28.443293539999999</v>
       </c>
     </row>
-    <row r="427" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="427" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A427" t="s">
         <v>9</v>
       </c>
@@ -19097,7 +19099,7 @@
         <v>29.123306410000001</v>
       </c>
     </row>
-    <row r="428" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="428" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A428" t="s">
         <v>9</v>
       </c>
@@ -19126,7 +19128,7 @@
         <v>28.069369630000001</v>
       </c>
     </row>
-    <row r="429" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="429" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A429" t="s">
         <v>9</v>
       </c>
@@ -19155,7 +19157,7 @@
         <v>28.159572010000002</v>
       </c>
     </row>
-    <row r="430" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="430" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A430" t="s">
         <v>9</v>
       </c>
@@ -19184,7 +19186,7 @@
         <v>28.598293739999999</v>
       </c>
     </row>
-    <row r="431" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="431" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A431" t="s">
         <v>9</v>
       </c>
@@ -19213,7 +19215,7 @@
         <v>28.56352446</v>
       </c>
     </row>
-    <row r="432" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="432" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A432" t="s">
         <v>9</v>
       </c>
@@ -19242,7 +19244,7 @@
         <v>29.004577560000001</v>
       </c>
     </row>
-    <row r="433" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="433" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A433" t="s">
         <v>9</v>
       </c>
@@ -19271,7 +19273,7 @@
         <v>29.16602279</v>
       </c>
     </row>
-    <row r="434" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="434" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A434" t="s">
         <v>9</v>
       </c>
@@ -19300,7 +19302,7 @@
         <v>29.02969173</v>
       </c>
     </row>
-    <row r="435" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="435" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A435" t="s">
         <v>9</v>
       </c>
@@ -19329,7 +19331,7 @@
         <v>29.050571170000001</v>
       </c>
     </row>
-    <row r="436" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="436" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A436" t="s">
         <v>9</v>
       </c>
@@ -19358,7 +19360,7 @@
         <v>27.298829820000002</v>
       </c>
     </row>
-    <row r="437" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="437" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A437" t="s">
         <v>9</v>
       </c>
@@ -19387,7 +19389,7 @@
         <v>27.34440609</v>
       </c>
     </row>
-    <row r="438" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="438" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A438" t="s">
         <v>9</v>
       </c>
@@ -19416,7 +19418,7 @@
         <v>27.56786469</v>
       </c>
     </row>
-    <row r="439" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="439" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A439" t="s">
         <v>9</v>
       </c>
@@ -19445,7 +19447,7 @@
         <v>28.525404930000001</v>
       </c>
     </row>
-    <row r="440" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="440" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A440" t="s">
         <v>9</v>
       </c>
@@ -19474,7 +19476,7 @@
         <v>27.945167900000001</v>
       </c>
     </row>
-    <row r="441" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="441" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A441" t="s">
         <v>9</v>
       </c>
@@ -19503,7 +19505,7 @@
         <v>28.8259513</v>
       </c>
     </row>
-    <row r="442" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="442" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A442" t="s">
         <v>9</v>
       </c>
@@ -19532,7 +19534,7 @@
         <v>28.848142920000001</v>
       </c>
     </row>
-    <row r="443" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="443" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A443" t="s">
         <v>9</v>
       </c>
@@ -19561,7 +19563,7 @@
         <v>28.867671519999998</v>
       </c>
     </row>
-    <row r="444" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="444" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A444" t="s">
         <v>9</v>
       </c>
@@ -19590,7 +19592,7 @@
         <v>28.785360950000001</v>
       </c>
     </row>
-    <row r="445" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="445" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A445" t="s">
         <v>9</v>
       </c>
@@ -19619,7 +19621,7 @@
         <v>25.601116189999999</v>
       </c>
     </row>
-    <row r="446" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="446" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A446" t="s">
         <v>9</v>
       </c>
@@ -19648,7 +19650,7 @@
         <v>23.796534650000002</v>
       </c>
     </row>
-    <row r="447" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="447" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A447" t="s">
         <v>9</v>
       </c>
@@ -19677,7 +19679,7 @@
         <v>25.439452930000002</v>
       </c>
     </row>
-    <row r="448" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="448" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A448" t="s">
         <v>9</v>
       </c>
@@ -19706,7 +19708,7 @@
         <v>23.599463320000002</v>
       </c>
     </row>
-    <row r="449" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="449" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A449" t="s">
         <v>9</v>
       </c>
@@ -19735,7 +19737,7 @@
         <v>22.628663</v>
       </c>
     </row>
-    <row r="450" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="450" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A450" t="s">
         <v>9</v>
       </c>
@@ -19764,7 +19766,7 @@
         <v>22.59713503</v>
       </c>
     </row>
-    <row r="451" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="451" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A451" t="s">
         <v>9</v>
       </c>
@@ -19793,7 +19795,7 @@
         <v>23.257300040000001</v>
       </c>
     </row>
-    <row r="452" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="452" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A452" t="s">
         <v>9</v>
       </c>
@@ -19822,7 +19824,7 @@
         <v>26.106890669999999</v>
       </c>
     </row>
-    <row r="453" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="453" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A453" t="s">
         <v>9</v>
       </c>
@@ -19851,7 +19853,7 @@
         <v>26.82248465</v>
       </c>
     </row>
-    <row r="454" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="454" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A454" t="s">
         <v>9</v>
       </c>
@@ -19880,7 +19882,7 @@
         <v>26.272839579999999</v>
       </c>
     </row>
-    <row r="455" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="455" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A455" t="s">
         <v>9</v>
       </c>
@@ -19909,7 +19911,7 @@
         <v>26.793969709999999</v>
       </c>
     </row>
-    <row r="456" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="456" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A456" t="s">
         <v>9</v>
       </c>
@@ -19938,7 +19940,7 @@
         <v>27.481561190000001</v>
       </c>
     </row>
-    <row r="457" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="457" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A457" t="s">
         <v>9</v>
       </c>
@@ -19967,7 +19969,7 @@
         <v>27.55233935</v>
       </c>
     </row>
-    <row r="458" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="458" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A458" t="s">
         <v>9</v>
       </c>
@@ -19996,7 +19998,7 @@
         <v>27.65597159</v>
       </c>
     </row>
-    <row r="459" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="459" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A459" t="s">
         <v>9</v>
       </c>
@@ -20025,7 +20027,7 @@
         <v>27.534141529999999</v>
       </c>
     </row>
-    <row r="460" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="460" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A460" t="s">
         <v>9</v>
       </c>
@@ -20054,7 +20056,7 @@
         <v>27.333992980000001</v>
       </c>
     </row>
-    <row r="461" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="461" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A461" t="s">
         <v>9</v>
       </c>
@@ -20083,7 +20085,7 @@
         <v>28.940280430000001</v>
       </c>
     </row>
-    <row r="462" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="462" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A462" t="s">
         <v>9</v>
       </c>
@@ -20112,7 +20114,7 @@
         <v>28.085977339999999</v>
       </c>
     </row>
-    <row r="463" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="463" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A463" t="s">
         <v>9</v>
       </c>
@@ -20141,7 +20143,7 @@
         <v>26.651226569999999</v>
       </c>
     </row>
-    <row r="464" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="464" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A464" t="s">
         <v>9</v>
       </c>
@@ -20170,7 +20172,7 @@
         <v>26.07154568</v>
       </c>
     </row>
-    <row r="465" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="465" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A465" t="s">
         <v>9</v>
       </c>
@@ -20199,7 +20201,7 @@
         <v>27.516480640000001</v>
       </c>
     </row>
-    <row r="466" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="466" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A466" t="s">
         <v>9</v>
       </c>
@@ -20228,7 +20230,7 @@
         <v>27.493750049999999</v>
       </c>
     </row>
-    <row r="467" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="467" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A467" t="s">
         <v>9</v>
       </c>
@@ -20257,7 +20259,7 @@
         <v>27.29607347</v>
       </c>
     </row>
-    <row r="468" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="468" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A468" t="s">
         <v>9</v>
       </c>
@@ -20286,7 +20288,7 @@
         <v>15.29799581</v>
       </c>
     </row>
-    <row r="469" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="469" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A469" t="s">
         <v>9</v>
       </c>
@@ -20315,7 +20317,7 @@
         <v>28.930896059999998</v>
       </c>
     </row>
-    <row r="470" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="470" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A470" t="s">
         <v>9</v>
       </c>
@@ -20344,7 +20346,7 @@
         <v>28.744326740000002</v>
       </c>
     </row>
-    <row r="471" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="471" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A471" t="s">
         <v>9</v>
       </c>
@@ -20373,7 +20375,7 @@
         <v>28.861616680000001</v>
       </c>
     </row>
-    <row r="472" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="472" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A472" t="s">
         <v>9</v>
       </c>
@@ -20402,7 +20404,7 @@
         <v>29.056543000000001</v>
       </c>
     </row>
-    <row r="473" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="473" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A473" t="s">
         <v>9</v>
       </c>
@@ -20431,7 +20433,7 @@
         <v>30.306178330000002</v>
       </c>
     </row>
-    <row r="474" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="474" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A474" t="s">
         <v>9</v>
       </c>
@@ -20460,7 +20462,7 @@
         <v>15.388876829999999</v>
       </c>
     </row>
-    <row r="475" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="475" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A475" t="s">
         <v>9</v>
       </c>
@@ -20489,7 +20491,7 @@
         <v>22.365857510000001</v>
       </c>
     </row>
-    <row r="476" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="476" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A476" t="s">
         <v>9</v>
       </c>
@@ -20518,7 +20520,7 @@
         <v>25.234624449999998</v>
       </c>
     </row>
-    <row r="477" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="477" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A477" t="s">
         <v>9</v>
       </c>
@@ -20547,7 +20549,7 @@
         <v>24.690773140000001</v>
       </c>
     </row>
-    <row r="478" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="478" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A478" t="s">
         <v>9</v>
       </c>
@@ -20576,7 +20578,7 @@
         <v>27.285491090000001</v>
       </c>
     </row>
-    <row r="479" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="479" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A479" t="s">
         <v>9</v>
       </c>
@@ -20605,7 +20607,7 @@
         <v>28.392519960000001</v>
       </c>
     </row>
-    <row r="480" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="480" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A480" t="s">
         <v>9</v>
       </c>
@@ -20634,7 +20636,7 @@
         <v>26.174780169999998</v>
       </c>
     </row>
-    <row r="481" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="481" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A481" t="s">
         <v>9</v>
       </c>
@@ -20663,7 +20665,7 @@
         <v>23.015731809999998</v>
       </c>
     </row>
-    <row r="482" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="482" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A482" t="s">
         <v>9</v>
       </c>
@@ -20692,7 +20694,7 @@
         <v>26.739187489999999</v>
       </c>
     </row>
-    <row r="483" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="483" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A483" t="s">
         <v>9</v>
       </c>
@@ -20721,7 +20723,7 @@
         <v>28.28384999</v>
       </c>
     </row>
-    <row r="484" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="484" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A484" t="s">
         <v>9</v>
       </c>
@@ -20750,7 +20752,7 @@
         <v>17.08422191</v>
       </c>
     </row>
-    <row r="485" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="485" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A485" t="s">
         <v>9</v>
       </c>
@@ -20779,7 +20781,7 @@
         <v>16.520030640000002</v>
       </c>
     </row>
-    <row r="486" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="486" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A486" t="s">
         <v>9</v>
       </c>
@@ -20808,7 +20810,7 @@
         <v>22.607630650000001</v>
       </c>
     </row>
-    <row r="487" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="487" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A487" t="s">
         <v>9</v>
       </c>
@@ -20837,7 +20839,7 @@
         <v>19.277279</v>
       </c>
     </row>
-    <row r="488" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="488" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A488" t="s">
         <v>9</v>
       </c>
@@ -20866,7 +20868,7 @@
         <v>21.995218650000002</v>
       </c>
     </row>
-    <row r="489" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="489" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A489" t="s">
         <v>9</v>
       </c>
@@ -20895,7 +20897,7 @@
         <v>22.433076249999999</v>
       </c>
     </row>
-    <row r="490" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="490" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A490" t="s">
         <v>9</v>
       </c>
@@ -20924,7 +20926,7 @@
         <v>21.373140379999999</v>
       </c>
     </row>
-    <row r="491" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="491" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A491" t="s">
         <v>9</v>
       </c>
@@ -20953,7 +20955,7 @@
         <v>20.161026440000001</v>
       </c>
     </row>
-    <row r="492" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="492" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A492" t="s">
         <v>9</v>
       </c>
@@ -20982,7 +20984,7 @@
         <v>18.932524189999999</v>
       </c>
     </row>
-    <row r="493" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="493" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A493" t="s">
         <v>9</v>
       </c>
@@ -21011,7 +21013,7 @@
         <v>18.44947749</v>
       </c>
     </row>
-    <row r="494" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="494" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A494" t="s">
         <v>9</v>
       </c>
@@ -21040,7 +21042,7 @@
         <v>18.825647549999999</v>
       </c>
     </row>
-    <row r="495" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="495" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A495" t="s">
         <v>9</v>
       </c>
@@ -21069,7 +21071,7 @@
         <v>19.082021619999999</v>
       </c>
     </row>
-    <row r="496" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="496" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A496" t="s">
         <v>9</v>
       </c>
@@ -21098,7 +21100,7 @@
         <v>22.087580620000001</v>
       </c>
     </row>
-    <row r="497" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="497" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A497" t="s">
         <v>9</v>
       </c>
@@ -21127,7 +21129,7 @@
         <v>21.34885061</v>
       </c>
     </row>
-    <row r="498" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="498" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A498" t="s">
         <v>9</v>
       </c>
@@ -21156,7 +21158,7 @@
         <v>20.88721481</v>
       </c>
     </row>
-    <row r="499" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="499" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A499" t="s">
         <v>9</v>
       </c>
@@ -21185,7 +21187,7 @@
         <v>19.64591982</v>
       </c>
     </row>
-    <row r="500" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="500" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A500" t="s">
         <v>9</v>
       </c>
@@ -21214,7 +21216,7 @@
         <v>20.931446619999999</v>
       </c>
     </row>
-    <row r="501" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="501" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A501" t="s">
         <v>9</v>
       </c>
@@ -21243,7 +21245,7 @@
         <v>20.287983530000002</v>
       </c>
     </row>
-    <row r="502" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="502" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A502" t="s">
         <v>9</v>
       </c>
@@ -21272,7 +21274,7 @@
         <v>21.371788280000001</v>
       </c>
     </row>
-    <row r="503" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="503" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A503" t="s">
         <v>9</v>
       </c>
@@ -21301,7 +21303,7 @@
         <v>22.161564370000001</v>
       </c>
     </row>
-    <row r="504" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="504" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A504" t="s">
         <v>9</v>
       </c>
@@ -21330,7 +21332,7 @@
         <v>19.872388430000001</v>
       </c>
     </row>
-    <row r="505" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="505" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A505" t="s">
         <v>9</v>
       </c>
@@ -21359,7 +21361,7 @@
         <v>20.784282900000001</v>
       </c>
     </row>
-    <row r="506" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="506" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A506" t="s">
         <v>9</v>
       </c>
@@ -21388,7 +21390,7 @@
         <v>21.829130320000001</v>
       </c>
     </row>
-    <row r="507" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="507" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A507" t="s">
         <v>9</v>
       </c>
@@ -21417,7 +21419,7 @@
         <v>20.013055309999999</v>
       </c>
     </row>
-    <row r="508" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="508" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A508" t="s">
         <v>9</v>
       </c>
@@ -21446,7 +21448,7 @@
         <v>17.795724249999999</v>
       </c>
     </row>
-    <row r="509" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="509" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A509" t="s">
         <v>9</v>
       </c>
@@ -21475,7 +21477,7 @@
         <v>18.550424670000002</v>
       </c>
     </row>
-    <row r="510" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="510" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A510" t="s">
         <v>9</v>
       </c>
@@ -21504,7 +21506,7 @@
         <v>18.230667220000001</v>
       </c>
     </row>
-    <row r="511" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="511" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A511" t="s">
         <v>9</v>
       </c>
@@ -21533,7 +21535,7 @@
         <v>18.05889462</v>
       </c>
     </row>
-    <row r="512" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="512" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A512" t="s">
         <v>9</v>
       </c>
@@ -21562,7 +21564,7 @@
         <v>19.086763600000001</v>
       </c>
     </row>
-    <row r="513" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="513" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A513" t="s">
         <v>9</v>
       </c>
@@ -21591,7 +21593,7 @@
         <v>18.81702452</v>
       </c>
     </row>
-    <row r="514" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="514" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A514" t="s">
         <v>9</v>
       </c>
@@ -21620,7 +21622,7 @@
         <v>18.545925530000002</v>
       </c>
     </row>
-    <row r="515" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="515" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A515" t="s">
         <v>9</v>
       </c>
@@ -21649,7 +21651,7 @@
         <v>17.65788903</v>
       </c>
     </row>
-    <row r="516" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="516" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A516" t="s">
         <v>9</v>
       </c>
@@ -21678,7 +21680,7 @@
         <v>18.391553640000001</v>
       </c>
     </row>
-    <row r="517" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="517" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A517" t="s">
         <v>9</v>
       </c>
@@ -21707,7 +21709,7 @@
         <v>17.102548429999999</v>
       </c>
     </row>
-    <row r="518" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="518" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A518" t="s">
         <v>9</v>
       </c>
@@ -21736,7 +21738,7 @@
         <v>18.23152176</v>
       </c>
     </row>
-    <row r="519" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="519" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A519" t="s">
         <v>9</v>
       </c>
@@ -21765,7 +21767,7 @@
         <v>17.914710240000002</v>
       </c>
     </row>
-    <row r="520" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="520" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A520" t="s">
         <v>9</v>
       </c>

</xml_diff>